<commit_message>
Allow text to be case insensitive
</commit_message>
<xml_diff>
--- a/data-raw/NZ ethnicity standard classification concordance.xlsx
+++ b/data-raw/NZ ethnicity standard classification concordance.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\uoc\jwilliman\3 Biostats\Resources\Data\Refs\Ethnicity\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://otagouni-my.sharepoint.com/personal/wiljo32p_registry_otago_ac_nz/Documents/MyFiles/2 Gits/ethnicNZ/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_B98B2062B1C1B3AA46EA0442E574D56FD7583A78" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9F05E6C-77FB-4889-BB1B-B50AA27CA274}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11850"/>
+    <workbookView xWindow="-26070" yWindow="3135" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="wbUQokQtCaYnPOB8" sheetId="1" r:id="rId1"/>
@@ -1899,7 +1900,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2216,7 +2217,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E339"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>